<commit_message>
Show the excluded-documents count as a number, not money
On the Summary sheet the COUNTA cell inherited column B's GBP format, so
39 excluded documents read as £39.00. The cell now has its own whole-
number format, with a test. The Excel fixture workbook is regenerated;
its tables are unchanged.
</commit_message>
<xml_diff>
--- a/excel/fixture/aged_debt_fixture.xlsx
+++ b/excel/fixture/aged_debt_fixture.xlsx
@@ -448,7 +448,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -463,6 +463,9 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1443,7 +1446,7 @@
       <c r="A10" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="10">
         <f>COUNTA(Unresolved!$B$2:$B$2)</f>
         <v>0</v>
       </c>
@@ -1466,7 +1469,7 @@
     <col min="5" max="5" width="34.7109375" customWidth="1"/>
     <col min="6" max="6" width="27.7109375" customWidth="1"/>
     <col min="7" max="7" width="18.7109375" customWidth="1"/>
-    <col min="8" max="9" width="13.7109375" style="10" customWidth="1"/>
+    <col min="8" max="9" width="13.7109375" style="11" customWidth="1"/>
     <col min="10" max="10" width="12.7109375" customWidth="1"/>
     <col min="11" max="11" width="11.7109375" customWidth="1"/>
     <col min="12" max="12" width="13.7109375" style="1" customWidth="1"/>
@@ -1544,10 +1547,10 @@
       <c r="G2" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="10">
+      <c r="H2" s="11">
         <v>46275</v>
       </c>
-      <c r="I2" s="10">
+      <c r="I2" s="11">
         <v>46305</v>
       </c>
       <c r="J2" t="s">
@@ -1588,10 +1591,10 @@
       <c r="G3" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="11">
         <v>46274</v>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="11">
         <v>46304</v>
       </c>
       <c r="J3" t="s">
@@ -1632,10 +1635,10 @@
       <c r="G4" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="10">
+      <c r="H4" s="11">
         <v>46245</v>
       </c>
-      <c r="I4" s="10">
+      <c r="I4" s="11">
         <v>46275</v>
       </c>
       <c r="J4" t="s">
@@ -1676,10 +1679,10 @@
       <c r="G5" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="10">
+      <c r="H5" s="11">
         <v>46244</v>
       </c>
-      <c r="I5" s="10">
+      <c r="I5" s="11">
         <v>46274</v>
       </c>
       <c r="J5" t="s">
@@ -1720,10 +1723,10 @@
       <c r="G6" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="10">
+      <c r="H6" s="11">
         <v>46215</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="11">
         <v>46245</v>
       </c>
       <c r="J6" t="s">
@@ -1764,10 +1767,10 @@
       <c r="G7" t="s">
         <v>42</v>
       </c>
-      <c r="H7" s="10">
+      <c r="H7" s="11">
         <v>46214</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I7" s="11">
         <v>46244</v>
       </c>
       <c r="J7" t="s">
@@ -1808,10 +1811,10 @@
       <c r="G8" t="s">
         <v>46</v>
       </c>
-      <c r="H8" s="10">
+      <c r="H8" s="11">
         <v>46185</v>
       </c>
-      <c r="I8" s="10">
+      <c r="I8" s="11">
         <v>46215</v>
       </c>
       <c r="J8" t="s">
@@ -1852,10 +1855,10 @@
       <c r="G9" t="s">
         <v>50</v>
       </c>
-      <c r="H9" s="10">
+      <c r="H9" s="11">
         <v>46184</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="11">
         <v>46214</v>
       </c>
       <c r="J9" t="s">
@@ -1896,10 +1899,10 @@
       <c r="G10" t="s">
         <v>54</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="11">
         <v>46306</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="11">
         <v>46336</v>
       </c>
       <c r="J10" t="s">
@@ -1940,10 +1943,10 @@
       <c r="G11" t="s">
         <v>59</v>
       </c>
-      <c r="H11" s="10">
+      <c r="H11" s="11">
         <v>46285</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="11">
         <v>46315</v>
       </c>
       <c r="J11" t="s">
@@ -1984,10 +1987,10 @@
       <c r="G12" t="s">
         <v>64</v>
       </c>
-      <c r="H12" s="10">
+      <c r="H12" s="11">
         <v>46266</v>
       </c>
-      <c r="I12" s="10">
+      <c r="I12" s="11">
         <v>46266</v>
       </c>
       <c r="K12" t="s">
@@ -2028,10 +2031,10 @@
       <c r="G13" t="s">
         <v>67</v>
       </c>
-      <c r="H13" s="10">
+      <c r="H13" s="11">
         <v>46307</v>
       </c>
-      <c r="I13" s="10">
+      <c r="I13" s="11">
         <v>46307</v>
       </c>
       <c r="K13" t="s">
@@ -2072,10 +2075,10 @@
       <c r="G14" t="s">
         <v>70</v>
       </c>
-      <c r="H14" s="10">
+      <c r="H14" s="11">
         <v>46280</v>
       </c>
-      <c r="I14" s="10">
+      <c r="I14" s="11">
         <v>46280</v>
       </c>
       <c r="K14" t="s">
@@ -2109,7 +2112,7 @@
   <cols>
     <col min="1" max="1" width="27.7109375" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" style="10" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" style="11" customWidth="1"/>
     <col min="4" max="5" width="13.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="12.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.7109375" style="1" customWidth="1"/>
@@ -2170,7 +2173,7 @@
       <c r="B2" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="11">
         <v>46305</v>
       </c>
       <c r="D2" s="1">
@@ -2214,7 +2217,7 @@
       <c r="B3" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="11">
         <v>46304</v>
       </c>
       <c r="D3" s="1">
@@ -2258,7 +2261,7 @@
       <c r="B4" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="11">
         <v>46275</v>
       </c>
       <c r="D4" s="1">
@@ -2302,7 +2305,7 @@
       <c r="B5" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="11">
         <v>46274</v>
       </c>
       <c r="D5" s="1">
@@ -2346,7 +2349,7 @@
       <c r="B6" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="11">
         <v>46245</v>
       </c>
       <c r="D6" s="1">
@@ -2390,7 +2393,7 @@
       <c r="B7" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="11">
         <v>46244</v>
       </c>
       <c r="D7" s="1">
@@ -2434,7 +2437,7 @@
       <c r="B8" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="11">
         <v>46215</v>
       </c>
       <c r="D8" s="1">
@@ -2478,7 +2481,7 @@
       <c r="B9" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="11">
         <v>46214</v>
       </c>
       <c r="D9" s="1">
@@ -2522,7 +2525,7 @@
       <c r="B10" t="s">
         <v>59</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="11">
         <v>46315</v>
       </c>
       <c r="D10" s="1">
@@ -2575,7 +2578,7 @@
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
     <col min="2" max="2" width="17.7109375" customWidth="1"/>
     <col min="3" max="3" width="27.7109375" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" style="10" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="11" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2606,7 +2609,7 @@
       <c r="C2" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="11">
         <v>46296</v>
       </c>
       <c r="E2" s="1">
@@ -2623,7 +2626,7 @@
       <c r="C3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="11">
         <v>46300</v>
       </c>
       <c r="E3" s="1">
@@ -2640,7 +2643,7 @@
       <c r="C4" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="11">
         <v>46306</v>
       </c>
       <c r="E4" s="1">
@@ -2657,7 +2660,7 @@
       <c r="C5" t="s">
         <v>58</v>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="11">
         <v>46295</v>
       </c>
       <c r="E5" s="1">
@@ -2674,7 +2677,7 @@
       <c r="C6" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="11">
         <v>46235</v>
       </c>
       <c r="E6" s="1">

</xml_diff>